<commit_message>
feat(ms-4.5): parameterize spectrum and spectrogram analysis
</commit_message>
<xml_diff>
--- a/docs/development/开发需求追踪矩阵.xlsx
+++ b/docs/development/开发需求追踪矩阵.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求总表" sheetId="1" r:id="Rb7ac1f8f387b463d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-页面" sheetId="2" r:id="R277b1237baa94a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-接口" sheetId="3" r:id="Rce512f377e7f40d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-测试" sheetId="4" r:id="Re51ffee540544a4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-里程碑" sheetId="5" r:id="R21be843da52b4964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-基础库" sheetId="6" r:id="R2c707a1f7f194af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-目标应用" sheetId="7" r:id="R78c05585c22f40f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺口与冲突" sheetId="8" r:id="R577e310defc74eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="9" r:id="Rd3a414ab7bf94bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="10" r:id="Ra73b8122771446d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求总表" sheetId="1" r:id="Rf9c5fb24ee824e6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-页面" sheetId="2" r:id="R1773a389df1e4807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-接口" sheetId="3" r:id="Rabc6f01d65814e9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-测试" sheetId="4" r:id="Re90d504a122c48cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-里程碑" sheetId="5" r:id="Ra19e599b921348ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-基础库" sheetId="6" r:id="R855bcd4aaf364070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="需求-目标应用" sheetId="7" r:id="R8e041e00b7b84723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺口与冲突" sheetId="8" r:id="R70ec88c4ab754a5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统计" sheetId="9" r:id="Rc9c9927e260848ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="10" r:id="R627cfb30ab094a6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="164" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="23">
+  <x:fonts count="25">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -149,6 +149,16 @@
       <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="宋体"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="宋体"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color theme="1"/>
+      <x:name val="Microsoft YaHei"/>
     </x:font>
   </x:fonts>
   <x:fills count="34">
@@ -319,7 +329,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="14">
     <x:border/>
     <x:border>
       <x:bottom style="thin">
@@ -408,6 +418,23 @@
       </x:top>
       <x:bottom style="double">
         <x:color theme="4"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="hair"/>
+    </x:border>
+    <x:border>
+      <x:top style="hair"/>
+      <x:bottom style="hair">
+        <x:color rgb="FFE3EAF0"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="hair">
+        <x:color rgb="FFE3EAF0"/>
+      </x:top>
+      <x:bottom style="hair">
+        <x:color rgb="FFE3EAF0"/>
       </x:bottom>
     </x:border>
   </x:borders>
@@ -558,7 +585,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="5">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -571,6 +598,25 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -18243,104 +18289,104 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200"/>
-      <x:c r="C200" t="str">
+      <x:c r="B200" s="14"/>
+      <x:c r="C200" s="14" t="str">
         <x:v>频谱结果平滑参数化</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>频谱支持滑动平均、高斯和 Savitzky-Golay 平滑；原始未平滑结果保留，纯平滑变化不重跑 FFT。</x:v>
       </x:c>
-      <x:c r="E200" t="str">
+      <x:c r="E200" s="14" t="str">
         <x:v>基础库/应用组合</x:v>
       </x:c>
-      <x:c r="F200" t="str">
+      <x:c r="F200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G200" t="str">
+      <x:c r="G200" s="14" t="str">
         <x:v>MS-4.5 任务文档</x:v>
       </x:c>
-      <x:c r="H200" t="str">
+      <x:c r="H200" s="14" t="str">
         <x:v>三种平滑真实改变显示结果；原始值可追溯；平滑专用缓存失效和数值测试通过。</x:v>
       </x:c>
-      <x:c r="I200" t="str">
+      <x:c r="I200" s="14" t="str">
         <x:v>UI-P03-001</x:v>
       </x:c>
-      <x:c r="J200" t="str">
+      <x:c r="J200" s="14" t="str">
         <x:v>API-DSP-001</x:v>
       </x:c>
-      <x:c r="K200" t="str">
+      <x:c r="K200" s="14" t="str">
         <x:v>TC-ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="L200" t="str">
+      <x:c r="L200" s="14" t="str">
         <x:v>MS-4.5</x:v>
       </x:c>
-      <x:c r="M200" t="str">
+      <x:c r="M200" s="14" t="str">
         <x:v>SignalDSP、SignalVisualization</x:v>
       </x:c>
-      <x:c r="N200" t="str">
+      <x:c r="N200" s="14" t="str">
         <x:v>Signal Studio</x:v>
       </x:c>
-      <x:c r="O200" t="str">
+      <x:c r="O200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
-      <x:c r="P200" t="str">
+      <x:c r="P200" s="14" t="str">
         <x:v>MS-4.5 独立提交</x:v>
       </x:c>
-      <x:c r="Q200" t="str">
+      <x:c r="Q200" s="14" t="str">
         <x:v>数值、缓存、持久化、UI 与 CPU/CUDA 后端一致性门禁通过</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201"/>
-      <x:c r="C201" t="str">
+      <x:c r="B201" s="15"/>
+      <x:c r="C201" s="15" t="str">
         <x:v>时频图平滑参数化</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>STFT 支持频率维高斯和时间维指数平滑；原始未平滑矩阵保留，纯平滑变化不重跑 STFT。</x:v>
       </x:c>
-      <x:c r="E201" t="str">
+      <x:c r="E201" s="15" t="str">
         <x:v>基础库/应用组合</x:v>
       </x:c>
-      <x:c r="F201" t="str">
+      <x:c r="F201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="G201" t="str">
+      <x:c r="G201" s="15" t="str">
         <x:v>MS-4.5 任务文档</x:v>
       </x:c>
-      <x:c r="H201" t="str">
+      <x:c r="H201" s="15" t="str">
         <x:v>频率维和时间维平滑真实改变时频结果；原始矩阵可追溯；最小失效和数值测试通过。</x:v>
       </x:c>
-      <x:c r="I201" t="str">
+      <x:c r="I201" s="15" t="str">
         <x:v>UI-P03-001</x:v>
       </x:c>
-      <x:c r="J201" t="str">
+      <x:c r="J201" s="15" t="str">
         <x:v>API-DSP-001</x:v>
       </x:c>
-      <x:c r="K201" t="str">
+      <x:c r="K201" s="15" t="str">
         <x:v>TC-ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="L201" t="str">
+      <x:c r="L201" s="15" t="str">
         <x:v>MS-4.5</x:v>
       </x:c>
-      <x:c r="M201" t="str">
+      <x:c r="M201" s="15" t="str">
         <x:v>SignalDSP、SignalVisualization</x:v>
       </x:c>
-      <x:c r="N201" t="str">
+      <x:c r="N201" s="15" t="str">
         <x:v>Signal Studio</x:v>
       </x:c>
-      <x:c r="O201" t="str">
+      <x:c r="O201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
-      <x:c r="P201" t="str">
+      <x:c r="P201" s="15" t="str">
         <x:v>MS-4.5 独立提交</x:v>
       </x:c>
-      <x:c r="Q201" t="str">
+      <x:c r="Q201" s="15" t="str">
         <x:v>数值、缓存、持久化、UI 与 CPU/CUDA 后端一致性门禁通过</x:v>
       </x:c>
     </x:row>
@@ -21994,30 +22040,30 @@
       </x:c>
     </x:row>
     <x:row r="162">
-      <x:c r="A162" t="str">
+      <x:c r="A162" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B162" t="str">
+      <x:c r="B162" s="14" t="str">
         <x:v>UI-P03-001</x:v>
       </x:c>
-      <x:c r="C162" t="str">
+      <x:c r="C162" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D162" t="str">
+      <x:c r="D162" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="163">
-      <x:c r="A163" t="str">
+      <x:c r="A163" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B163" t="str">
+      <x:c r="B163" s="15" t="str">
         <x:v>UI-P03-001</x:v>
       </x:c>
-      <x:c r="C163" t="str">
+      <x:c r="C163" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D163" t="str">
+      <x:c r="D163" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
@@ -26415,30 +26461,30 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200" t="str">
+      <x:c r="B200" s="14" t="str">
         <x:v>API-DSP-001</x:v>
       </x:c>
-      <x:c r="C200" t="str">
+      <x:c r="C200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201" t="str">
+      <x:c r="B201" s="15" t="str">
         <x:v>API-DSP-001</x:v>
       </x:c>
-      <x:c r="C201" t="str">
+      <x:c r="C201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
@@ -30836,30 +30882,30 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200" t="str">
+      <x:c r="B200" s="14" t="str">
         <x:v>TC-ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="C200" t="str">
+      <x:c r="C200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201" t="str">
+      <x:c r="B201" s="15" t="str">
         <x:v>TC-ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="C201" t="str">
+      <x:c r="C201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
@@ -35257,30 +35303,30 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200" t="str">
+      <x:c r="B200" s="14" t="str">
         <x:v>MS-4.5</x:v>
       </x:c>
-      <x:c r="C200" t="str">
+      <x:c r="C200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201" t="str">
+      <x:c r="B201" s="15" t="str">
         <x:v>MS-4.5</x:v>
       </x:c>
-      <x:c r="C201" t="str">
+      <x:c r="C201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
@@ -39678,30 +39724,30 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200" t="str">
+      <x:c r="B200" s="14" t="str">
         <x:v>SignalDSP、SignalVisualization</x:v>
       </x:c>
-      <x:c r="C200" t="str">
+      <x:c r="C200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201" t="str">
+      <x:c r="B201" s="15" t="str">
         <x:v>SignalDSP、SignalVisualization</x:v>
       </x:c>
-      <x:c r="C201" t="str">
+      <x:c r="C201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
@@ -44099,30 +44145,30 @@
       </x:c>
     </x:row>
     <x:row r="200">
-      <x:c r="A200" t="str">
+      <x:c r="A200" s="14" t="str">
         <x:v>ENH-SPEC-001</x:v>
       </x:c>
-      <x:c r="B200" t="str">
+      <x:c r="B200" s="14" t="str">
         <x:v>Signal Studio</x:v>
       </x:c>
-      <x:c r="C200" t="str">
+      <x:c r="C200" s="14" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D200" t="str">
+      <x:c r="D200" s="14" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>
     <x:row r="201">
-      <x:c r="A201" t="str">
+      <x:c r="A201" s="15" t="str">
         <x:v>ENH-SPEC-002</x:v>
       </x:c>
-      <x:c r="B201" t="str">
+      <x:c r="B201" s="15" t="str">
         <x:v>Signal Studio</x:v>
       </x:c>
-      <x:c r="C201" t="str">
+      <x:c r="C201" s="15" t="str">
         <x:v>P0</x:v>
       </x:c>
-      <x:c r="D201" t="str">
+      <x:c r="D201" s="15" t="str">
         <x:v>已验收</x:v>
       </x:c>
     </x:row>

</xml_diff>